<commit_message>
chore: add health check route and update production API URL
</commit_message>
<xml_diff>
--- a/backend/Solar_Load_Template.xlsx
+++ b/backend/Solar_Load_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>Consumer Name</t>
   </si>
@@ -26,12 +26,6 @@
   </si>
   <si>
     <t>Connection Type</t>
-  </si>
-  <si>
-    <t>Contract Demand (KVA) :</t>
-  </si>
-  <si>
-    <t>Solar Pannel used</t>
   </si>
   <si>
     <t>Sr.No</t>
@@ -74,9 +68,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.000000000"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -110,12 +103,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFF4B084"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4B084"/>
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -143,37 +136,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -514,14 +501,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:J30"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="4" width="20" customWidth="1"/>
-    <col min="5" max="6" width="15" customWidth="1"/>
-    <col min="7" max="8" width="20" customWidth="1"/>
-    <col min="9" max="10" width="15" customWidth="1"/>
+    <col min="3" max="10" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -559,285 +543,260 @@
       <c r="D5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="5"/>
-    </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="6" t="s">
+      <c r="D8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="E8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="F8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="G8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>2</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>3</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>4</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>6</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>7</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>8</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>9</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
         <v>10</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="B18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
         <v>11</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B9" s="4">
-        <v>2</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-    </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B10" s="4">
-        <v>3</v>
-      </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B11" s="4">
-        <v>4</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-    </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="4">
-        <v>5</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="4">
-        <v>6</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="4">
-        <v>7</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="4">
-        <v>8</v>
-      </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-    </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B16" s="4">
-        <v>9</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B17" s="4">
-        <v>10</v>
-      </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B18" s="4">
-        <v>11</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B19" s="4">
+      <c r="B19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
         <v>12</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B20" s="4">
-        <v>13</v>
-      </c>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="4">
-        <v>14</v>
-      </c>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="7">
-        <f>AVERAGE(D9:D20)</f>
-      </c>
-      <c r="H22" s="7">
-        <f>AVERAGE(H9:H20)</f>
-      </c>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="8">
-        <f>D22/106.06</f>
-      </c>
-      <c r="H23" s="8">
-        <f>H22/106.06</f>
-      </c>
+      <c r="B20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="8">
-        <f>D23/0.6</f>
-      </c>
-      <c r="H24" s="8">
-        <f>H23/0.6</f>
+        <v>10</v>
+      </c>
+      <c r="D24" s="4">
+        <f>IFERROR(AVERAGE(D9:D20), 0)</f>
+      </c>
+      <c r="H24" s="4">
+        <f>IFERROR(AVERAGE(H9:H20), 0)</f>
       </c>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="9">
-        <f>ROUND(D24*0.6, 1)</f>
-      </c>
-      <c r="H25" s="9">
-        <f>ROUND(H24*0.6, 1)</f>
+        <v>11</v>
+      </c>
+      <c r="D25" s="4">
+        <f>D24/106.06</f>
+      </c>
+      <c r="H25" s="4">
+        <f>H24/106.06</f>
       </c>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="4">
+        <f>D25/0.6</f>
+      </c>
+      <c r="H26" s="4">
+        <f>H25/0.6</f>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="5">
+        <f>ROUND(D26*0.6, 1)</f>
+      </c>
+      <c r="H27" s="5">
+        <f>ROUND(H26*0.6, 1)</f>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="6">
+        <f>ROUNDUP(D26, 0)</f>
+      </c>
+      <c r="H28" s="6">
+        <f>ROUNDUP(H26, 0)</f>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="8">
+        <f>D27+H27</f>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="10">
-        <f>ROUNDUP(D24, 0)</f>
-      </c>
-      <c r="H26" s="10">
-        <f>ROUNDUP(H24, 0)</f>
-      </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="2">
-        <f>D25+H25</f>
-      </c>
-    </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D30" s="2">
-        <f>D26+H26</f>
+      <c r="D30" s="8">
+        <f>D28+H28</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: restructure excel columns and fix pdf processing crash
</commit_message>
<xml_diff>
--- a/backend/Solar_Load_Template.xlsx
+++ b/backend/Solar_Load_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="19">
   <si>
     <t>Consumer Name</t>
   </si>
@@ -26,6 +26,12 @@
   </si>
   <si>
     <t>Connection Type</t>
+  </si>
+  <si>
+    <t>Contract Demand (KVA) :</t>
+  </si>
+  <si>
+    <t>Solar Pannel used</t>
   </si>
   <si>
     <t>Sr.No</t>
@@ -501,9 +507,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J30"/>
+  <dimension ref="B1:J30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="10" width="15" customWidth="1"/>
   </cols>
@@ -543,40 +550,54 @@
       <c r="D5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="D6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>7</v>
-      </c>
       <c r="I8" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="2">
         <v>1</v>
       </c>
-      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -585,11 +606,11 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="2">
         <v>2</v>
       </c>
-      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -598,11 +619,11 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="2">
         <v>3</v>
       </c>
-      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -611,11 +632,11 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="2">
         <v>4</v>
       </c>
-      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -624,11 +645,11 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="2">
         <v>5</v>
       </c>
-      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -637,11 +658,11 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="2">
         <v>6</v>
       </c>
-      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
@@ -650,11 +671,11 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="2">
         <v>7</v>
       </c>
-      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -663,11 +684,11 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
         <v>8</v>
       </c>
-      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -676,11 +697,11 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
         <v>9</v>
       </c>
-      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
@@ -689,11 +710,11 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="2">
         <v>10</v>
       </c>
-      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -702,11 +723,11 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="2">
         <v>11</v>
       </c>
-      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
@@ -715,11 +736,11 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="2">
         <v>12</v>
       </c>
-      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
@@ -730,7 +751,7 @@
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D24" s="4">
         <f>IFERROR(AVERAGE(D9:D20), 0)</f>
@@ -741,7 +762,7 @@
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D25" s="4">
         <f>D24/106.06</f>
@@ -752,7 +773,7 @@
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D26" s="4">
         <f>D25/0.6</f>
@@ -763,7 +784,7 @@
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D27" s="5">
         <f>ROUND(D26*0.6, 1)</f>
@@ -774,7 +795,7 @@
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D28" s="6">
         <f>ROUNDUP(D26, 0)</f>
@@ -785,7 +806,7 @@
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D29" s="8">
         <f>D27+H27</f>
@@ -793,7 +814,7 @@
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D30" s="8">
         <f>D28+H28</f>

</xml_diff>